<commit_message>
Correction parsing caractères parasites et montants
</commit_message>
<xml_diff>
--- a/excel test.xlsx
+++ b/excel test.xlsx
@@ -1,43 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mael.dekeuwer\Documents\perso\benchmark\Old\suivi_dep\dev\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{659CBEFE-F343-4C1B-BEDB-00EF9F73521A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11805" xr2:uid="{609DB3AA-D15C-4CCB-A695-1B7BB2973125}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11805" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
+    <sheet name="Feuil1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Operations" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -55,22 +48,82 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -370,10 +423,282 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83D1ED68-8E89-471D-A918-63D16261DEAF}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Tiers</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Libellé brut</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Montant</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Source PDF</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Date import</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>ID opération</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Mr Bricolage Sainte 11/10</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Carte X1840 Mr Bricolage Sainte 11/10</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>-6.9</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Releve n 002 du 04-11-2025_CCHQ 30018815253 MONSIEUR DEKEUWER MAEL.pdf</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>46161</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>40248099cdc8230d</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Suravenir</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Prlv Suravenir</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>-250</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Releve n 002 du 04-11-2025_CCHQ 30018815253 MONSIEUR DEKEUWER MAEL.pdf</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>46161</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>22ff995ed5456e2a</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>** Offre Essentiel</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Cotis ** Offre Essentiel</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>-8</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Releve n 002 du 04-11-2025_CCHQ 30018815253 MONSIEUR DEKEUWER MAEL.pdf</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>46161</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>286f09bbd74ee5ff</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>des camelias Saint-d 25/10</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Carte X1840 des camelias Saint-d 25/10</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>-12.89</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Releve n 002 du 04-11-2025_CCHQ 30018815253 MONSIEUR DEKEUWER MAEL.pdf</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>46161</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>db68324543c47da4</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paierie Departementale Reunion 2</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Virement Paierie Departementale Reunion 2</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>542.4299999999999</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Releve n 002 du 04-11-2025_CCHQ 30018815253 MONSIEUR DEKEUWER MAEL.pdf</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>46161</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>c10c3779bd46a22e</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Sumup *maison tikok 30/10</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Carte X1840 Sumup *maison tikok 30/10</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>-12</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Releve n 002 du 04-11-2025_CCHQ 30018815253 MONSIEUR DEKEUWER MAEL.pdf</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>46161</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>40aaf1883ab2570e</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Dekeuwer Mael</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Virement Web Dekeuwer Mael</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>-700</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Releve n 002 du 04-11-2025_CCHQ 30018815253 MONSIEUR DEKEUWER MAEL.pdf</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>46161</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>d14b5bc55ff2a0b7</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>